<commit_message>
finish feature export billing
</commit_message>
<xml_diff>
--- a/templates/record_billing.xlsx
+++ b/templates/record_billing.xlsx
@@ -8,14 +8,26 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/congdat/Developer/lab-admin-go/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C31DEC91-87EA-5D41-8DE9-D0C728F0F900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED87A533-5830-C647-AC13-656A46798E61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6340" yWindow="1640" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="181029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -37,9 +49,6 @@
     <t>Họ tên</t>
   </si>
   <si>
-    <t>Tuổi</t>
-  </si>
-  <si>
     <t>Địa chỉ</t>
   </si>
   <si>
@@ -62,6 +71,9 @@
   </si>
   <si>
     <t>Nguyễn Công Mẫn</t>
+  </si>
+  <si>
+    <t>Năm sinh</t>
   </si>
 </sst>
 </file>
@@ -167,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -195,14 +207,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -478,22 +487,18 @@
       <c r="E5" s="2"/>
     </row>
     <row r="6" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="3"/>
+    </row>
+    <row r="7" spans="1:5" ht="13" x14ac:dyDescent="0.15">
+      <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-    </row>
-    <row r="7" spans="1:5" ht="13" x14ac:dyDescent="0.15">
-      <c r="A7" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
     </row>
@@ -505,25 +510,25 @@
       <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" s="14" t="s">
+      <c r="A9" s="13" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="C9" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="D9" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="E9" s="14" t="s">
         <v>10</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="C12" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
@@ -550,7 +555,7 @@
     </row>
     <row r="17" spans="3:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="C17" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>

</xml_diff>